<commit_message>
feat: polish dashboard experience and add delivery docs
</commit_message>
<xml_diff>
--- a/sample_data/campus_resource_dataset.xlsx
+++ b/sample_data/campus_resource_dataset.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working_green_campus\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F683893-C778-47F5-868F-030437AA5230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08569F27-5648-43AA-A082-4EFE03AC842F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,13 @@
     <sheet name="solar" sheetId="1" r:id="rId1"/>
     <sheet name="energy" sheetId="2" r:id="rId2"/>
     <sheet name="water" sheetId="3" r:id="rId3"/>
-    <sheet name="waste" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="28">
   <si>
     <t>date</t>
   </si>
@@ -107,9 +106,6 @@
   </si>
   <si>
     <t>water_kl</t>
-  </si>
-  <si>
-    <t>waste_kg</t>
   </si>
 </sst>
 </file>
@@ -1256,267 +1252,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:C23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3">
-        <v>920</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4">
-        <v>940</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5">
-        <v>960</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6">
-        <v>980</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8">
-        <v>1020</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9">
-        <v>1040</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C10">
-        <v>1060</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11">
-        <v>1080</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" t="s">
-        <v>4</v>
-      </c>
-      <c r="C12">
-        <v>1100</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B13" t="s">
-        <v>4</v>
-      </c>
-      <c r="C13">
-        <v>1120</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14" t="s">
-        <v>4</v>
-      </c>
-      <c r="C14">
-        <v>1140</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>17</v>
-      </c>
-      <c r="B15" t="s">
-        <v>4</v>
-      </c>
-      <c r="C15">
-        <v>1160</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16" t="s">
-        <v>4</v>
-      </c>
-      <c r="C16">
-        <v>1180</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17" t="s">
-        <v>4</v>
-      </c>
-      <c r="C17">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18" t="s">
-        <v>4</v>
-      </c>
-      <c r="C18">
-        <v>1220</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19" t="s">
-        <v>4</v>
-      </c>
-      <c r="C19">
-        <v>1240</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>22</v>
-      </c>
-      <c r="B20" t="s">
-        <v>4</v>
-      </c>
-      <c r="C20">
-        <v>1260</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>23</v>
-      </c>
-      <c r="B21" t="s">
-        <v>4</v>
-      </c>
-      <c r="C21">
-        <v>1280</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>24</v>
-      </c>
-      <c r="B22" t="s">
-        <v>4</v>
-      </c>
-      <c r="C22">
-        <v>1300</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>25</v>
-      </c>
-      <c r="B23" t="s">
-        <v>4</v>
-      </c>
-      <c r="C23">
-        <v>1320</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>